<commit_message>
Faster input because of skips
</commit_message>
<xml_diff>
--- a/data/database/shopgraph_purchase_history.xlsx
+++ b/data/database/shopgraph_purchase_history.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imported Receipts" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Purchase History'!$A$1:$O$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Purchase History'!$A$1:$O$99</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,9 +27,9 @@
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="mmm yyyy"/>
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="172" formatCode="mm/dd/yyyy hh:mm"/>
+    <numFmt numFmtId="170" formatCode="mm/dd/yyyy hh:mm"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -265,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -354,7 +354,8 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3468,7 +3469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="27" min="1" max="1"/>
@@ -7094,6 +7095,12 @@
       <c r="M73" s="1" t="n">
         <v>3.48</v>
       </c>
+      <c r="N73" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="O73" s="1" t="n">
+        <v>1.76</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1">
@@ -7141,6 +7148,12 @@
       <c r="K74" s="1" t="n">
         <v>16.92</v>
       </c>
+      <c r="L74" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="M74" s="1" t="n">
+        <v>17.72</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1">
@@ -7565,8 +7578,784 @@
         <v>5</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="1">
+        <f>SUM(K84,M84,O84)</f>
+        <v/>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Nature's Bakery Gluten Free Raspberry Fig Bars in Twin pack Box, 20z Each 36 shopped Qty1</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K84" s="1" t="n">
+        <v>5.97</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1">
+        <f>SUM(K85,M85,O85)</f>
+        <v/>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Mahatma Jasmine Rice, Thai Fragrant Long Grain Rice, Gluten Free, 80 oz Bag (5 lbs</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K85" s="1" t="n">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1">
+        <f>SUM(K86,M86,O86)</f>
+        <v/>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Hillshire Farm Ultra Thin Oven Roasted Turkey Breast Lunchmeat, 16 oz Plastic Tub, Refrigerated</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K86" s="1" t="n">
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1">
+        <f>SUM(K87,M87,O87)</f>
+        <v/>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Hebrew National 100% Kosher Beef Franks, Hot Dogs, 10.3 oz 6 Count</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K87" s="1" t="n">
+        <v>5.74</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1">
+        <f>SUM(K88,M88,O88)</f>
+        <v/>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Dave's Killer Bread Organic Oats &amp; Blues Regular Size Loaf, 25 oz, USDA Organic</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K88" s="1" t="n">
+        <v>5.98</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1">
+        <f>SUM(K89,M89,O89)</f>
+        <v/>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Birds Eye Steamfresh Sweet Peas, Frozen Vegetables, 10 oz. Bag</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K89" s="1" t="n">
+        <v>1.27</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1">
+        <f>SUM(K90,M90,O90)</f>
+        <v/>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Cabot Creamery 4 Cheese Mexican Shredded Cheddar Cheese 2 lb (Refrigerated</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K90" s="1" t="n">
+        <v>11.93</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1">
+        <f>SUM(K91,M91,O91)</f>
+        <v/>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Ziploc Brand Slider Gallon Freezer Food Storage Bags, School Supplies, with Power Shield Technology, 40 Count</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K91" s="1" t="n">
+        <v>7.98</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1">
+        <f>SUM(K92,M92,O92)</f>
+        <v/>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Ziploc Brand Freezer Food Storage Bags, School Supplies, with Grip 'n Seal Technology, Zipper, Quart, 50 Count</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K92" s="1" t="n">
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1">
+        <f>SUM(K93,M93,O93)</f>
+        <v/>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Fresh Mini Cucumbers, 16 oz</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K93" s="1" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1">
+        <f>SUM(K94,M94,O94)</f>
+        <v/>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2 pack) Yehuda Sabbath Candles,12ct</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K94" s="1" t="n">
+        <v>3.16</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1">
+        <f>SUM(K95,M95,O95)</f>
+        <v/>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Fresh Yellow Squash, Each 11 weight adjusted aty1</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K95" s="1" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="M95" s="1" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1">
+        <f>SUM(K96,M96,O96)</f>
+        <v/>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Fresh Zucchini, Each 11 weight adjusted aty1</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Zucchini</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K96" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="M96" s="1" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1">
+        <f>SUM(K97,M97,O97)</f>
+        <v/>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Fresh Whole Red Onion, Each</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K97" s="1" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L97" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="M97" s="1" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1">
+        <f>SUM(K98,M98,O98)</f>
+        <v/>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Fresh Tomato on the Vine, Bag (1.9 lbs/Bag Est.) 11 weight adjusted Qty1</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K98" s="1" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1">
+        <f>SUM(K99,M99,O99)</f>
+        <v/>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Fresh Banana, Each 11 weight adjusted Qty7</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K99" s="1" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="L99" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="M99" s="1" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O83"/>
+  <autoFilter ref="A1:O99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12138,7 +12927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="27" min="1" max="1"/>
@@ -12273,8 +13062,44 @@
       <c r="C7" s="2" t="n">
         <v>46241</v>
       </c>
-      <c r="D7" s="56" t="n">
-        <v>46262.59873947963</v>
+      <c r="D7" s="57" t="n">
+        <v>46262.59873947917</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>081326_Walmart_0_raw_ocr.json</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>46262.65887388889</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>081326_Walmart_0_B_raw_ocr.json</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D9" s="57" t="n">
+        <v>46262.66004273877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
can clean everything now
</commit_message>
<xml_diff>
--- a/data/database/shopgraph_purchase_history.xlsx
+++ b/data/database/shopgraph_purchase_history.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imported Receipts" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Purchase History'!$A$1:$O$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Purchase History'!$A$1:$S$106</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3469,7 +3469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O99"/>
+  <dimension ref="A1:S106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="27" min="1" max="1"/>
@@ -3487,6 +3487,10 @@
     <col width="14" customWidth="1" style="27" min="13" max="13"/>
     <col width="14" customWidth="1" style="27" min="14" max="14"/>
     <col width="14" customWidth="1" style="27" min="15" max="15"/>
+    <col width="14" customWidth="1" style="27" min="16" max="16"/>
+    <col width="14" customWidth="1" style="27" min="17" max="17"/>
+    <col width="14" customWidth="1" style="27" min="18" max="18"/>
+    <col width="14" customWidth="1" style="27" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3561,10 +3565,30 @@
           <t>Price 3</t>
         </is>
       </c>
+      <c r="P1" s="52" t="inlineStr">
+        <is>
+          <t>Date 4</t>
+        </is>
+      </c>
+      <c r="Q1" s="52" t="inlineStr">
+        <is>
+          <t>Price 4</t>
+        </is>
+      </c>
+      <c r="R1" s="52" t="inlineStr">
+        <is>
+          <t>Date 5</t>
+        </is>
+      </c>
+      <c r="S1" s="52" t="inlineStr">
+        <is>
+          <t>Price 5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>SUM(K2,M2,O2)</f>
+        <f>SUM(K2,M2,O2,Q2,S2)</f>
         <v/>
       </c>
       <c r="C2" t="inlineStr">
@@ -3611,7 +3635,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <f>SUM(K3,M3,O3)</f>
+        <f>SUM(K3,M3,O3,Q3,S3)</f>
         <v/>
       </c>
       <c r="C3" t="inlineStr">
@@ -3658,7 +3682,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <f>SUM(K4,M4,O4)</f>
+        <f>SUM(K4,M4,O4,Q4,S4)</f>
         <v/>
       </c>
       <c r="C4" t="inlineStr">
@@ -3705,7 +3729,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <f>SUM(K5,M5,O5)</f>
+        <f>SUM(K5,M5,O5,Q5,S5)</f>
         <v/>
       </c>
       <c r="C5" t="inlineStr">
@@ -3758,7 +3782,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <f>SUM(K6,M6,O6)</f>
+        <f>SUM(K6,M6,O6,Q6,S6)</f>
         <v/>
       </c>
       <c r="C6" t="inlineStr">
@@ -3805,7 +3829,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <f>SUM(K7,M7,O7)</f>
+        <f>SUM(K7,M7,O7,Q7,S7)</f>
         <v/>
       </c>
       <c r="C7" t="inlineStr">
@@ -3864,7 +3888,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <f>SUM(K8,M8,O8)</f>
+        <f>SUM(K8,M8,O8,Q8,S8)</f>
         <v/>
       </c>
       <c r="C8" t="inlineStr">
@@ -3911,7 +3935,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <f>SUM(K9,M9,O9)</f>
+        <f>SUM(K9,M9,O9,Q9,S9)</f>
         <v/>
       </c>
       <c r="C9" t="inlineStr">
@@ -3958,7 +3982,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <f>SUM(K10,M10,O10)</f>
+        <f>SUM(K10,M10,O10,Q10,S10)</f>
         <v/>
       </c>
       <c r="C10" t="inlineStr">
@@ -4005,7 +4029,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <f>SUM(K11,M11,O11)</f>
+        <f>SUM(K11,M11,O11,Q11,S11)</f>
         <v/>
       </c>
       <c r="C11" t="inlineStr">
@@ -4052,7 +4076,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <f>SUM(K12,M12,O12)</f>
+        <f>SUM(K12,M12,O12,Q12,S12)</f>
         <v/>
       </c>
       <c r="C12" t="inlineStr">
@@ -4099,7 +4123,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <f>SUM(K13,M13,O13)</f>
+        <f>SUM(K13,M13,O13,Q13,S13)</f>
         <v/>
       </c>
       <c r="C13" t="inlineStr">
@@ -4146,7 +4170,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <f>SUM(K14,M14,O14)</f>
+        <f>SUM(K14,M14,O14,Q14,S14)</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
@@ -4193,7 +4217,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <f>SUM(K15,M15,O15)</f>
+        <f>SUM(K15,M15,O15,Q15,S15)</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
@@ -4240,7 +4264,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <f>SUM(K16,M16,O16)</f>
+        <f>SUM(K16,M16,O16,Q16,S16)</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr">
@@ -4287,7 +4311,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <f>SUM(K17,M17,O17)</f>
+        <f>SUM(K17,M17,O17,Q17,S17)</f>
         <v/>
       </c>
       <c r="C17" t="inlineStr">
@@ -4334,7 +4358,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <f>SUM(K18,M18,O18)</f>
+        <f>SUM(K18,M18,O18,Q18,S18)</f>
         <v/>
       </c>
       <c r="C18" t="inlineStr">
@@ -4381,7 +4405,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <f>SUM(K19,M19,O19)</f>
+        <f>SUM(K19,M19,O19,Q19,S19)</f>
         <v/>
       </c>
       <c r="C19" t="inlineStr">
@@ -4428,7 +4452,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <f>SUM(K20,M20,O20)</f>
+        <f>SUM(K20,M20,O20,Q20,S20)</f>
         <v/>
       </c>
       <c r="C20" t="inlineStr">
@@ -4475,7 +4499,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <f>SUM(K21,M21,O21)</f>
+        <f>SUM(K21,M21,O21,Q21,S21)</f>
         <v/>
       </c>
       <c r="C21" t="inlineStr">
@@ -4522,7 +4546,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <f>SUM(K22,M22,O22)</f>
+        <f>SUM(K22,M22,O22,Q22,S22)</f>
         <v/>
       </c>
       <c r="C22" t="inlineStr">
@@ -4569,7 +4593,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <f>SUM(K23,M23,O23)</f>
+        <f>SUM(K23,M23,O23,Q23,S23)</f>
         <v/>
       </c>
       <c r="C23" t="inlineStr">
@@ -4616,7 +4640,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <f>SUM(K24,M24,O24)</f>
+        <f>SUM(K24,M24,O24,Q24,S24)</f>
         <v/>
       </c>
       <c r="C24" t="inlineStr">
@@ -4663,7 +4687,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1">
-        <f>SUM(K25,M25,O25)</f>
+        <f>SUM(K25,M25,O25,Q25,S25)</f>
         <v/>
       </c>
       <c r="C25" t="inlineStr">
@@ -4710,7 +4734,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1">
-        <f>SUM(K26,M26,O26)</f>
+        <f>SUM(K26,M26,O26,Q26,S26)</f>
         <v/>
       </c>
       <c r="C26" t="inlineStr">
@@ -4763,7 +4787,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1">
-        <f>SUM(K27,M27,O27)</f>
+        <f>SUM(K27,M27,O27,Q27,S27)</f>
         <v/>
       </c>
       <c r="C27" t="inlineStr">
@@ -4810,7 +4834,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1">
-        <f>SUM(K28,M28,O28)</f>
+        <f>SUM(K28,M28,O28,Q28,S28)</f>
         <v/>
       </c>
       <c r="C28" t="inlineStr">
@@ -4863,7 +4887,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1">
-        <f>SUM(K29,M29,O29)</f>
+        <f>SUM(K29,M29,O29,Q29,S29)</f>
         <v/>
       </c>
       <c r="C29" t="inlineStr">
@@ -4916,7 +4940,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1">
-        <f>SUM(K30,M30,O30)</f>
+        <f>SUM(K30,M30,O30,Q30,S30)</f>
         <v/>
       </c>
       <c r="C30" t="inlineStr">
@@ -4963,7 +4987,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1">
-        <f>SUM(K31,M31,O31)</f>
+        <f>SUM(K31,M31,O31,Q31,S31)</f>
         <v/>
       </c>
       <c r="C31" t="inlineStr">
@@ -5010,7 +5034,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1">
-        <f>SUM(K32,M32,O32)</f>
+        <f>SUM(K32,M32,O32,Q32,S32)</f>
         <v/>
       </c>
       <c r="C32" t="inlineStr">
@@ -5057,7 +5081,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1">
-        <f>SUM(K33,M33,O33)</f>
+        <f>SUM(K33,M33,O33,Q33,S33)</f>
         <v/>
       </c>
       <c r="C33" t="inlineStr">
@@ -5104,7 +5128,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1">
-        <f>SUM(K34,M34,O34)</f>
+        <f>SUM(K34,M34,O34,Q34,S34)</f>
         <v/>
       </c>
       <c r="C34" t="inlineStr">
@@ -5151,7 +5175,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1">
-        <f>SUM(K35,M35,O35)</f>
+        <f>SUM(K35,M35,O35,Q35,S35)</f>
         <v/>
       </c>
       <c r="C35" t="inlineStr">
@@ -5198,7 +5222,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1">
-        <f>SUM(K36,M36,O36)</f>
+        <f>SUM(K36,M36,O36,Q36,S36)</f>
         <v/>
       </c>
       <c r="C36" t="inlineStr">
@@ -5245,7 +5269,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1">
-        <f>SUM(K37,M37,O37)</f>
+        <f>SUM(K37,M37,O37,Q37,S37)</f>
         <v/>
       </c>
       <c r="C37" t="inlineStr">
@@ -5292,7 +5316,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1">
-        <f>SUM(K38,M38,O38)</f>
+        <f>SUM(K38,M38,O38,Q38,S38)</f>
         <v/>
       </c>
       <c r="C38" t="inlineStr">
@@ -5339,7 +5363,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1">
-        <f>SUM(K39,M39,O39)</f>
+        <f>SUM(K39,M39,O39,Q39,S39)</f>
         <v/>
       </c>
       <c r="C39" t="inlineStr">
@@ -5386,7 +5410,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1">
-        <f>SUM(K40,M40,O40)</f>
+        <f>SUM(K40,M40,O40,Q40,S40)</f>
         <v/>
       </c>
       <c r="C40" t="inlineStr">
@@ -5439,7 +5463,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1">
-        <f>SUM(K41,M41,O41)</f>
+        <f>SUM(K41,M41,O41,Q41,S41)</f>
         <v/>
       </c>
       <c r="C41" t="inlineStr">
@@ -5486,7 +5510,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1">
-        <f>SUM(K42,M42,O42)</f>
+        <f>SUM(K42,M42,O42,Q42,S42)</f>
         <v/>
       </c>
       <c r="C42" t="inlineStr">
@@ -5533,7 +5557,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1">
-        <f>SUM(K43,M43,O43)</f>
+        <f>SUM(K43,M43,O43,Q43,S43)</f>
         <v/>
       </c>
       <c r="C43" t="inlineStr">
@@ -5580,7 +5604,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1">
-        <f>SUM(K44,M44,O44)</f>
+        <f>SUM(K44,M44,O44,Q44,S44)</f>
         <v/>
       </c>
       <c r="C44" t="inlineStr">
@@ -5627,7 +5651,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1">
-        <f>SUM(K45,M45,O45)</f>
+        <f>SUM(K45,M45,O45,Q45,S45)</f>
         <v/>
       </c>
       <c r="C45" t="inlineStr">
@@ -5674,7 +5698,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1">
-        <f>SUM(K46,M46,O46)</f>
+        <f>SUM(K46,M46,O46,Q46,S46)</f>
         <v/>
       </c>
       <c r="C46" t="inlineStr">
@@ -5721,7 +5745,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1">
-        <f>SUM(K47,M47,O47)</f>
+        <f>SUM(K47,M47,O47,Q47,S47)</f>
         <v/>
       </c>
       <c r="C47" t="inlineStr">
@@ -5768,7 +5792,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1">
-        <f>SUM(K48,M48,O48)</f>
+        <f>SUM(K48,M48,O48,Q48,S48)</f>
         <v/>
       </c>
       <c r="C48" t="inlineStr">
@@ -5815,7 +5839,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1">
-        <f>SUM(K49,M49,O49)</f>
+        <f>SUM(K49,M49,O49,Q49,S49)</f>
         <v/>
       </c>
       <c r="C49" t="inlineStr">
@@ -5862,7 +5886,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1">
-        <f>SUM(K50,M50,O50)</f>
+        <f>SUM(K50,M50,O50,Q50,S50)</f>
         <v/>
       </c>
       <c r="C50" t="inlineStr">
@@ -5909,7 +5933,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1">
-        <f>SUM(K51,M51,O51)</f>
+        <f>SUM(K51,M51,O51,Q51,S51)</f>
         <v/>
       </c>
       <c r="C51" t="inlineStr">
@@ -5962,7 +5986,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1">
-        <f>SUM(K52,M52,O52)</f>
+        <f>SUM(K52,M52,O52,Q52,S52)</f>
         <v/>
       </c>
       <c r="C52" t="inlineStr">
@@ -6015,7 +6039,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1">
-        <f>SUM(K53,M53,O53)</f>
+        <f>SUM(K53,M53,O53,Q53,S53)</f>
         <v/>
       </c>
       <c r="C53" t="inlineStr">
@@ -6068,7 +6092,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1">
-        <f>SUM(K54,M54,O54)</f>
+        <f>SUM(K54,M54,O54,Q54,S54)</f>
         <v/>
       </c>
       <c r="C54" t="inlineStr">
@@ -6115,7 +6139,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1">
-        <f>SUM(K55,M55,O55)</f>
+        <f>SUM(K55,M55,O55,Q55,S55)</f>
         <v/>
       </c>
       <c r="C55" t="inlineStr">
@@ -6168,7 +6192,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1">
-        <f>SUM(K56,M56,O56)</f>
+        <f>SUM(K56,M56,O56,Q56,S56)</f>
         <v/>
       </c>
       <c r="C56" t="inlineStr">
@@ -6221,7 +6245,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1">
-        <f>SUM(K57,M57,O57)</f>
+        <f>SUM(K57,M57,O57,Q57,S57)</f>
         <v/>
       </c>
       <c r="C57" t="inlineStr">
@@ -6274,7 +6298,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1">
-        <f>SUM(K58,M58,O58)</f>
+        <f>SUM(K58,M58,O58,Q58,S58)</f>
         <v/>
       </c>
       <c r="C58" t="inlineStr">
@@ -6321,7 +6345,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1">
-        <f>SUM(K59,M59,O59)</f>
+        <f>SUM(K59,M59,O59,Q59,S59)</f>
         <v/>
       </c>
       <c r="C59" t="inlineStr">
@@ -6368,7 +6392,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1">
-        <f>SUM(K60,M60,O60)</f>
+        <f>SUM(K60,M60,O60,Q60,S60)</f>
         <v/>
       </c>
       <c r="C60" t="inlineStr">
@@ -6421,7 +6445,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1">
-        <f>SUM(K61,M61,O61)</f>
+        <f>SUM(K61,M61,O61,Q61,S61)</f>
         <v/>
       </c>
       <c r="C61" t="inlineStr">
@@ -6474,7 +6498,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1">
-        <f>SUM(K62,M62,O62)</f>
+        <f>SUM(K62,M62,O62,Q62,S62)</f>
         <v/>
       </c>
       <c r="C62" t="inlineStr">
@@ -6521,7 +6545,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1">
-        <f>SUM(K63,M63,O63)</f>
+        <f>SUM(K63,M63,O63,Q63,S63)</f>
         <v/>
       </c>
       <c r="C63" t="inlineStr">
@@ -6574,7 +6598,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1">
-        <f>SUM(K64,M64,O64)</f>
+        <f>SUM(K64,M64,O64,Q64,S64)</f>
         <v/>
       </c>
       <c r="C64" t="inlineStr">
@@ -6627,7 +6651,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1">
-        <f>SUM(K65,M65,O65)</f>
+        <f>SUM(K65,M65,O65,Q65,S65)</f>
         <v/>
       </c>
       <c r="C65" t="inlineStr">
@@ -6680,7 +6704,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1">
-        <f>SUM(K66,M66,O66)</f>
+        <f>SUM(K66,M66,O66,Q66,S66)</f>
         <v/>
       </c>
       <c r="C66" t="inlineStr">
@@ -6733,7 +6757,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1">
-        <f>SUM(K67,M67,O67)</f>
+        <f>SUM(K67,M67,O67,Q67,S67)</f>
         <v/>
       </c>
       <c r="C67" t="inlineStr">
@@ -6780,7 +6804,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1">
-        <f>SUM(K68,M68,O68)</f>
+        <f>SUM(K68,M68,O68,Q68,S68)</f>
         <v/>
       </c>
       <c r="C68" t="inlineStr">
@@ -6833,7 +6857,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1">
-        <f>SUM(K69,M69,O69)</f>
+        <f>SUM(K69,M69,O69,Q69,S69)</f>
         <v/>
       </c>
       <c r="C69" t="inlineStr">
@@ -6886,7 +6910,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1">
-        <f>SUM(K70,M70,O70)</f>
+        <f>SUM(K70,M70,O70,Q70,S70)</f>
         <v/>
       </c>
       <c r="C70" t="inlineStr">
@@ -6945,7 +6969,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1">
-        <f>SUM(K71,M71,O71)</f>
+        <f>SUM(K71,M71,O71,Q71,S71)</f>
         <v/>
       </c>
       <c r="C71" t="inlineStr">
@@ -6998,7 +7022,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1">
-        <f>SUM(K72,M72,O72)</f>
+        <f>SUM(K72,M72,O72,Q72,S72)</f>
         <v/>
       </c>
       <c r="C72" t="inlineStr">
@@ -7045,7 +7069,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1">
-        <f>SUM(K73,M73,O73)</f>
+        <f>SUM(K73,M73,O73,Q73,S73)</f>
         <v/>
       </c>
       <c r="C73" t="inlineStr">
@@ -7101,10 +7125,22 @@
       <c r="O73" s="1" t="n">
         <v>1.76</v>
       </c>
+      <c r="P73" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="Q73" s="1" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="R73" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="S73" s="1" t="n">
+        <v>6.35</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1">
-        <f>SUM(K74,M74,O74)</f>
+        <f>SUM(K74,M74,O74,Q74,S74)</f>
         <v/>
       </c>
       <c r="C74" t="inlineStr">
@@ -7154,10 +7190,16 @@
       <c r="M74" s="1" t="n">
         <v>17.72</v>
       </c>
+      <c r="N74" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="O74" s="1" t="n">
+        <v>12.14</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1">
-        <f>SUM(K75,M75,O75)</f>
+        <f>SUM(K75,M75,O75,Q75,S75)</f>
         <v/>
       </c>
       <c r="C75" t="inlineStr">
@@ -7204,7 +7246,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1">
-        <f>SUM(K76,M76,O76)</f>
+        <f>SUM(K76,M76,O76,Q76,S76)</f>
         <v/>
       </c>
       <c r="C76" t="inlineStr">
@@ -7251,7 +7293,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1">
-        <f>SUM(K77,M77,O77)</f>
+        <f>SUM(K77,M77,O77,Q77,S77)</f>
         <v/>
       </c>
       <c r="C77" t="inlineStr">
@@ -7298,7 +7340,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1">
-        <f>SUM(K78,M78,O78)</f>
+        <f>SUM(K78,M78,O78,Q78,S78)</f>
         <v/>
       </c>
       <c r="C78" t="inlineStr">
@@ -7345,7 +7387,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1">
-        <f>SUM(K79,M79,O79)</f>
+        <f>SUM(K79,M79,O79,Q79,S79)</f>
         <v/>
       </c>
       <c r="C79" t="inlineStr">
@@ -7392,7 +7434,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1">
-        <f>SUM(K80,M80,O80)</f>
+        <f>SUM(K80,M80,O80,Q80,S80)</f>
         <v/>
       </c>
       <c r="C80" t="inlineStr">
@@ -7439,7 +7481,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1">
-        <f>SUM(K81,M81,O81)</f>
+        <f>SUM(K81,M81,O81,Q81,S81)</f>
         <v/>
       </c>
       <c r="C81" t="inlineStr">
@@ -7486,7 +7528,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1">
-        <f>SUM(K82,M82,O82)</f>
+        <f>SUM(K82,M82,O82,Q82,S82)</f>
         <v/>
       </c>
       <c r="C82" t="inlineStr">
@@ -7533,7 +7575,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1">
-        <f>SUM(K83,M83,O83)</f>
+        <f>SUM(K83,M83,O83,Q83,S83)</f>
         <v/>
       </c>
       <c r="C83" t="inlineStr">
@@ -7580,7 +7622,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1">
-        <f>SUM(K84,M84,O84)</f>
+        <f>SUM(K84,M84,O84,Q84,S84)</f>
         <v/>
       </c>
       <c r="C84" t="inlineStr">
@@ -7627,7 +7669,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1">
-        <f>SUM(K85,M85,O85)</f>
+        <f>SUM(K85,M85,O85,Q85,S85)</f>
         <v/>
       </c>
       <c r="C85" t="inlineStr">
@@ -7674,7 +7716,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1">
-        <f>SUM(K86,M86,O86)</f>
+        <f>SUM(K86,M86,O86,Q86,S86)</f>
         <v/>
       </c>
       <c r="C86" t="inlineStr">
@@ -7721,7 +7763,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1">
-        <f>SUM(K87,M87,O87)</f>
+        <f>SUM(K87,M87,O87,Q87,S87)</f>
         <v/>
       </c>
       <c r="C87" t="inlineStr">
@@ -7768,7 +7810,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1">
-        <f>SUM(K88,M88,O88)</f>
+        <f>SUM(K88,M88,O88,Q88,S88)</f>
         <v/>
       </c>
       <c r="C88" t="inlineStr">
@@ -7815,7 +7857,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1">
-        <f>SUM(K89,M89,O89)</f>
+        <f>SUM(K89,M89,O89,Q89,S89)</f>
         <v/>
       </c>
       <c r="C89" t="inlineStr">
@@ -7862,7 +7904,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1">
-        <f>SUM(K90,M90,O90)</f>
+        <f>SUM(K90,M90,O90,Q90,S90)</f>
         <v/>
       </c>
       <c r="C90" t="inlineStr">
@@ -7909,7 +7951,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1">
-        <f>SUM(K91,M91,O91)</f>
+        <f>SUM(K91,M91,O91,Q91,S91)</f>
         <v/>
       </c>
       <c r="C91" t="inlineStr">
@@ -7956,7 +7998,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1">
-        <f>SUM(K92,M92,O92)</f>
+        <f>SUM(K92,M92,O92,Q92,S92)</f>
         <v/>
       </c>
       <c r="C92" t="inlineStr">
@@ -8003,7 +8045,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1">
-        <f>SUM(K93,M93,O93)</f>
+        <f>SUM(K93,M93,O93,Q93,S93)</f>
         <v/>
       </c>
       <c r="C93" t="inlineStr">
@@ -8050,7 +8092,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1">
-        <f>SUM(K94,M94,O94)</f>
+        <f>SUM(K94,M94,O94,Q94,S94)</f>
         <v/>
       </c>
       <c r="C94" t="inlineStr">
@@ -8097,7 +8139,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1">
-        <f>SUM(K95,M95,O95)</f>
+        <f>SUM(K95,M95,O95,Q95,S95)</f>
         <v/>
       </c>
       <c r="C95" t="inlineStr">
@@ -8150,7 +8192,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1">
-        <f>SUM(K96,M96,O96)</f>
+        <f>SUM(K96,M96,O96,Q96,S96)</f>
         <v/>
       </c>
       <c r="C96" t="inlineStr">
@@ -8203,7 +8245,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1">
-        <f>SUM(K97,M97,O97)</f>
+        <f>SUM(K97,M97,O97,Q97,S97)</f>
         <v/>
       </c>
       <c r="C97" t="inlineStr">
@@ -8256,7 +8298,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1">
-        <f>SUM(K98,M98,O98)</f>
+        <f>SUM(K98,M98,O98,Q98,S98)</f>
         <v/>
       </c>
       <c r="C98" t="inlineStr">
@@ -8303,7 +8345,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1">
-        <f>SUM(K99,M99,O99)</f>
+        <f>SUM(K99,M99,O99,Q99,S99)</f>
         <v/>
       </c>
       <c r="C99" t="inlineStr">
@@ -8354,8 +8396,345 @@
         <v>1.76</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="1">
+        <f>SUM(K100,M100,O100,Q100,S100)</f>
+        <v/>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Command Heavy Duty Picture Hangers, Hold 20 tbs, Black, Damage-Free Hanging, 8 Pairs Adhesive Strips</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K100" s="1" t="n">
+        <v>28.54</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1">
+        <f>SUM(K101,M101,O101,Q101,S101)</f>
+        <v/>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Dove Men+Care Antiperspirant Deodorant Stick 72-Hour Sweat &amp; Odor Protection Clean Comfort Antiperspirant For Men</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1">
+        <f>SUM(K102,M102,O102,Q102,S102)</f>
+        <v/>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Dawn Ultra 11" Puff Glassware and Dish Cleaning Brush Wand with Sponge Head</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K102" s="1" t="n">
+        <v>4.46</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1">
+        <f>SUM(K103,M103,O103,Q103,S103)</f>
+        <v/>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Once Upon a Farm Organic Tractor Wheels Toddler Bar, Apple, Sweet Potato &amp; Spinach, 10ct</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K103" s="1" t="n">
+        <v>9.98</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1">
+        <f>SUM(K104,M104,O104,Q104,S104)</f>
+        <v/>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Weiman Granite &amp; Stone Disinfectant Cleaner &amp; Polish, 24 floz</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K104" s="1" t="n">
+        <v>6.24</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1">
+        <f>SUM(K105,M105,O105,Q105,S105)</f>
+        <v/>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Chobani Low-Fat Vanilla Greek Yogurt Mixed Berry On The Bottom, Hero Batch z 4PK</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K105" s="1" t="n">
+        <v>4.67</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1">
+        <f>SUM(K106,M106,O106,Q106,S106)</f>
+        <v/>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Fresh Banana, Each 4 weight adjusted aty4</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="K106" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L106" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="M106" s="1" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O99"/>
+  <autoFilter ref="A1:S106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12927,7 +13306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="27" min="1" max="1"/>
@@ -13099,7 +13478,25 @@
         <v>46247</v>
       </c>
       <c r="D9" s="57" t="n">
-        <v>46262.66004273877</v>
+        <v>46262.66004274305</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>082626_Walmart_0_raw_ocr.json</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>46262.67645812407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>